<commit_message>
[Data] Update xlsx files
</commit_message>
<xml_diff>
--- a/server/coach-infos.xlsx
+++ b/server/coach-infos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\samir\archifoot\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143B7441-422D-41D1-88EB-53EC9CCAB26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BA431E-21FB-4D26-9B2A-35DD09D9DE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="entraineurs" sheetId="1" r:id="rId1"/>
@@ -538,9 +538,6 @@
 En septembre 1991, il décrocha également le titre afro-asiatique, remporté en aller-retour face à l’Iran. Ce doublé reste l’un des plus grands exploits de l’histoire des Verts.</t>
   </si>
   <si>
-    <t>IGHIL Meziane</t>
-  </si>
-  <si>
     <t>12/01/1954</t>
   </si>
   <si>
@@ -556,9 +553,6 @@
 Le Hussein-déen revint ensuite à la tête de l’EN, cette fois en duo avec un technicien roumain, Piguela, mais la collaboration ne dura que trois matches.
 Ighil dirigea encore trois autres rencontres avant d’être écarté après une défaite à domicile contre la Tunisie.
 Il revint une nouvelle fois, à titre intérimaire, pour achever les matches de qualification Coupe du monde / CAN en juin 1995, rencontres sans enjeu puisque l’Algérie était déjà éliminée.</t>
-  </si>
-  <si>
-    <t>MEHDAOUI Abderahmane</t>
   </si>
   <si>
     <t>07/10/1949</t>
@@ -687,9 +681,6 @@
 La lourde défaite en Égypte (5–2), en éliminatoires du Mondial 2002, poussa la Fédération à limoger les deux hommes.</t>
   </si>
   <si>
-    <t>RADULESCU MIRCEA</t>
-  </si>
-  <si>
     <t>31/08/1941</t>
   </si>
   <si>
@@ -725,9 +716,6 @@
 Georges Leekens a mené une riche carrière d’entraîneur, aussi bien en club qu’en sélection. Il a exercé dans les principaux clubs belges et dirigé quatre équipes nationales : l’Algérie, la Belgique, la Tunisie et la Hongrie.</t>
   </si>
   <si>
-    <t>WASEIGE Robert</t>
-  </si>
-  <si>
     <t>26/08/1939</t>
   </si>
   <si>
@@ -775,9 +763,6 @@
 Sous sa direction, l’Algérie dispute néanmoins deux rencontres amicales de prestige en 2007, en Europe, face à deux grandes nations du football mondial : l’Argentine de Lionel Messi et le Brésil de Kaká. Les deux confrontations se soldent par des défaites honorables et étriquées de la sélection algérienne.</t>
   </si>
   <si>
-    <t>BENCHIKHA Abdelhak</t>
-  </si>
-  <si>
     <t>22/11/1963</t>
   </si>
   <si>
@@ -786,9 +771,6 @@
   <si>
     <t>Abdelhak Benchikha succède à Rabah Saâdane, démissionnaire. Toutefois, après la lourde défaite concédée face au Maroc (4-0) à Marrakech, lors du match retour des éliminatoires de la Coupe d’Afrique des nations 2013, il préfère mettre un terme à sa mission à la tête des Verts.
 Benchikha demeure néanmoins un entraîneur de grande valeur. Il a remporté plusieurs titres nationaux dans différents pays et s’est illustré sur la scène continentale, notamment en décrochant la Coupe de la CAF avec l’USM Alger. En reconnaissance de son parcours, il est désigné meilleur entraîneur du monde arabe en 2013.</t>
-  </si>
-  <si>
-    <t>HALILHODZIC Vahid</t>
   </si>
   <si>
     <t>15/05/1952</t>
@@ -856,9 +838,6 @@
     <t>Adjoint de Christian Gourcuff, Nabil Neghiz a dirigé un seul match à la tête de la sélection nationale : la rencontre disputée face aux Seychelles en juin 2016, dans le cadre des éliminatoires de la CAN 2017.
 Il est resté en poste comme entraîneur adjoint jusqu’en janvier 2017.
 En 2023, il fait son retour au sein des Verts pour seconder Vladimir Petković.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RAJEAC Milovan </t>
   </si>
   <si>
     <t>02/01/1954</t>
@@ -922,9 +901,6 @@
 Belmadi et Abdelhamid Kermali demeurent à ce jour les seuls sélectionneurs algériens vainqueurs de la Coupe d’Afrique des Nations, respectivement en 1990 et 2019.</t>
   </si>
   <si>
-    <t xml:space="preserve">PETKOVICH Vladimir </t>
-  </si>
-  <si>
     <t>Sarajevo</t>
   </si>
   <si>
@@ -937,9 +913,6 @@
     <t>En poste depuis depuis mars 2024, Vladilmir Pectovic a réussi à qualifier l’équipe nationale en coupe du Monde de 2026 et en coupe d’Afrique des nations 2025 . Dans la compétition africaine, il a franchi les matches du groupe et atteindre les 1/4 de finale. Ce qui lui a permis de poursuivre sa mission pour la phase finale de la coupe du monde.</t>
   </si>
   <si>
-    <t xml:space="preserve">CHERADI Rachid </t>
-  </si>
-  <si>
     <t xml:space="preserve">Cheraga </t>
   </si>
   <si>
@@ -1430,13 +1403,40 @@
   </si>
   <si>
     <t>1934/1983</t>
+  </si>
+  <si>
+    <t>Ighil Ali Meziane</t>
+  </si>
+  <si>
+    <t>Mehdaoui Abderrahmane</t>
+  </si>
+  <si>
+    <t>Rădulescu Mircea</t>
+  </si>
+  <si>
+    <t>Waseige Robert</t>
+  </si>
+  <si>
+    <t>Benchikha Abdelhak</t>
+  </si>
+  <si>
+    <t>Halilhodžić Vahid</t>
+  </si>
+  <si>
+    <t>Rajevac Milovan</t>
+  </si>
+  <si>
+    <t>Petković Vladimir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rachid Cherradi </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1480,6 +1480,12 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1519,7 +1525,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1527,11 +1533,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1558,6 +1579,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1956,7 +1980,7 @@
         <v>13</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>14</v>
@@ -1991,7 +2015,7 @@
         <v>22</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>439</v>
+        <v>430</v>
       </c>
       <c r="K2" s="15" t="s">
         <v>21</v>
@@ -2094,10 +2118,10 @@
         <v>19</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="K4" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -2144,7 +2168,7 @@
         <v>39</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>441</v>
+        <v>432</v>
       </c>
       <c r="K5" t="s">
         <v>44</v>
@@ -2197,10 +2221,10 @@
         <v>19</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>442</v>
+        <v>433</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -2300,7 +2324,7 @@
         <v>64</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="L8">
         <v>10</v>
@@ -2350,7 +2374,7 @@
         <v>71</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -2444,7 +2468,7 @@
         <v>84</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -2511,7 +2535,7 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="B13" s="5">
         <v>11441</v>
@@ -2538,7 +2562,7 @@
         <v>97</v>
       </c>
       <c r="K13" s="15" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -2779,7 +2803,7 @@
         <v>141</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="L18">
         <v>2</v>
@@ -2829,7 +2853,7 @@
         <v>149</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="L19">
         <v>10</v>
@@ -2879,7 +2903,7 @@
         <v>156</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="L20">
         <v>1</v>
@@ -2900,15 +2924,15 @@
         <v>157</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
-      <c r="A21" t="s">
+    <row r="21" spans="1:17" ht="15.75">
+      <c r="A21" s="16" t="s">
+        <v>434</v>
+      </c>
+      <c r="B21" t="s">
         <v>158</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>159</v>
-      </c>
-      <c r="C21" t="s">
-        <v>160</v>
       </c>
       <c r="D21" t="s">
         <v>39</v>
@@ -2917,7 +2941,7 @@
         <v>19</v>
       </c>
       <c r="J21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K21" t="s">
         <v>126</v>
@@ -2938,15 +2962,15 @@
         <v>6</v>
       </c>
       <c r="Q21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>163</v>
+        <v>435</v>
       </c>
       <c r="B22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>39</v>
@@ -2958,7 +2982,7 @@
         <v>19</v>
       </c>
       <c r="F22" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="G22" t="s">
         <v>39</v>
@@ -2967,7 +2991,7 @@
         <v>19</v>
       </c>
       <c r="J22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K22" t="s">
         <v>126</v>
@@ -2988,15 +3012,15 @@
         <v>27</v>
       </c>
       <c r="Q22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>39</v>
@@ -3008,10 +3032,10 @@
         <v>19</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K23" s="15" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="L23">
         <v>90</v>
@@ -3029,30 +3053,30 @@
         <v>0</v>
       </c>
       <c r="Q23" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" spans="1:17">
       <c r="A24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24" t="s">
+        <v>171</v>
+      </c>
+      <c r="C24" t="s">
         <v>172</v>
       </c>
-      <c r="B24" t="s">
+      <c r="D24" t="s">
         <v>173</v>
-      </c>
-      <c r="C24" t="s">
-        <v>174</v>
-      </c>
-      <c r="D24" t="s">
-        <v>175</v>
       </c>
       <c r="E24" t="s">
         <v>22</v>
       </c>
       <c r="J24" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K24" s="15" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="L24">
         <v>73</v>
@@ -3070,27 +3094,27 @@
         <v>19</v>
       </c>
       <c r="Q24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="25" spans="1:17">
       <c r="A25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" t="s">
+        <v>177</v>
+      </c>
+      <c r="C25" t="s">
         <v>178</v>
       </c>
-      <c r="B25" t="s">
-        <v>179</v>
-      </c>
-      <c r="C25" t="s">
-        <v>180</v>
-      </c>
       <c r="D25" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E25" t="s">
         <v>19</v>
       </c>
       <c r="F25" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G25" t="s">
         <v>77</v>
@@ -3099,7 +3123,7 @@
         <v>22</v>
       </c>
       <c r="K25" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -3117,30 +3141,30 @@
         <v>19</v>
       </c>
       <c r="Q25" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" t="s">
+        <v>182</v>
+      </c>
+      <c r="B26" t="s">
+        <v>183</v>
+      </c>
+      <c r="C26" t="s">
         <v>184</v>
       </c>
-      <c r="B26" t="s">
+      <c r="D26" t="s">
         <v>185</v>
-      </c>
-      <c r="C26" t="s">
-        <v>186</v>
-      </c>
-      <c r="D26" t="s">
-        <v>187</v>
       </c>
       <c r="E26" t="s">
         <v>94</v>
       </c>
       <c r="J26" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -3158,18 +3182,18 @@
         <v>3</v>
       </c>
       <c r="Q26" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" t="s">
+        <v>188</v>
+      </c>
+      <c r="B27" t="s">
+        <v>189</v>
+      </c>
+      <c r="C27" t="s">
         <v>190</v>
-      </c>
-      <c r="B27" t="s">
-        <v>191</v>
-      </c>
-      <c r="C27" t="s">
-        <v>192</v>
       </c>
       <c r="D27" t="s">
         <v>77</v>
@@ -3178,10 +3202,10 @@
         <v>22</v>
       </c>
       <c r="J27" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K27" s="15" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -3199,30 +3223,30 @@
         <v>0</v>
       </c>
       <c r="Q27" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" spans="1:17">
       <c r="A28" t="s">
+        <v>193</v>
+      </c>
+      <c r="B28" t="s">
+        <v>194</v>
+      </c>
+      <c r="C28" t="s">
         <v>195</v>
-      </c>
-      <c r="B28" t="s">
-        <v>196</v>
-      </c>
-      <c r="C28" t="s">
-        <v>197</v>
       </c>
       <c r="D28" t="s">
         <v>124</v>
       </c>
       <c r="E28" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="J28" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K28" s="15" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="L28">
         <v>3</v>
@@ -3240,15 +3264,15 @@
         <v>9</v>
       </c>
       <c r="Q28" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:17">
       <c r="A29" t="s">
-        <v>201</v>
+        <v>436</v>
       </c>
       <c r="B29" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C29" t="s">
         <v>93</v>
@@ -3260,10 +3284,10 @@
         <v>94</v>
       </c>
       <c r="J29" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="K29" s="15" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="L29">
         <v>0</v>
@@ -3281,30 +3305,30 @@
         <v>9</v>
       </c>
       <c r="Q29" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" t="s">
+        <v>203</v>
+      </c>
+      <c r="C30" t="s">
+        <v>204</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B30" t="s">
+      <c r="E30" t="s">
         <v>206</v>
       </c>
-      <c r="C30" t="s">
+      <c r="J30" t="s">
         <v>207</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="K30" t="s">
         <v>208</v>
-      </c>
-      <c r="E30" t="s">
-        <v>209</v>
-      </c>
-      <c r="J30" t="s">
-        <v>210</v>
-      </c>
-      <c r="K30" t="s">
-        <v>211</v>
       </c>
       <c r="L30">
         <v>3</v>
@@ -3322,39 +3346,39 @@
         <v>0</v>
       </c>
       <c r="Q30" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" spans="1:17">
       <c r="A31" t="s">
+        <v>437</v>
+      </c>
+      <c r="B31" t="s">
+        <v>210</v>
+      </c>
+      <c r="C31" t="s">
+        <v>211</v>
+      </c>
+      <c r="D31" t="s">
+        <v>212</v>
+      </c>
+      <c r="E31" t="s">
+        <v>206</v>
+      </c>
+      <c r="F31" t="s">
         <v>213</v>
       </c>
-      <c r="B31" t="s">
+      <c r="G31" t="s">
         <v>214</v>
       </c>
-      <c r="C31" t="s">
+      <c r="I31" t="s">
+        <v>206</v>
+      </c>
+      <c r="J31" t="s">
         <v>215</v>
       </c>
-      <c r="D31" t="s">
+      <c r="K31" t="s">
         <v>216</v>
-      </c>
-      <c r="E31" t="s">
-        <v>209</v>
-      </c>
-      <c r="F31" t="s">
-        <v>217</v>
-      </c>
-      <c r="G31" t="s">
-        <v>218</v>
-      </c>
-      <c r="I31" t="s">
-        <v>209</v>
-      </c>
-      <c r="J31" t="s">
-        <v>219</v>
-      </c>
-      <c r="K31" t="s">
-        <v>220</v>
       </c>
       <c r="L31">
         <v>0</v>
@@ -3372,30 +3396,30 @@
         <v>0</v>
       </c>
       <c r="Q31" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" spans="1:17">
       <c r="A32" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B32" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C32" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D32" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="E32" t="s">
         <v>22</v>
       </c>
       <c r="J32" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="K32" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="L32">
         <v>0</v>
@@ -3413,30 +3437,30 @@
         <v>0</v>
       </c>
       <c r="Q32" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="1:17">
       <c r="A33" t="s">
-        <v>229</v>
+        <v>438</v>
       </c>
       <c r="B33" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="C33" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D33" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E33" t="s">
         <v>19</v>
       </c>
       <c r="J33" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="K33" s="15" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="L33">
         <v>0</v>
@@ -3454,30 +3478,30 @@
         <v>0</v>
       </c>
       <c r="Q33" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34" spans="1:17">
       <c r="A34" t="s">
+        <v>439</v>
+      </c>
+      <c r="B34" t="s">
+        <v>228</v>
+      </c>
+      <c r="C34" t="s">
+        <v>229</v>
+      </c>
+      <c r="D34" t="s">
+        <v>230</v>
+      </c>
+      <c r="E34" t="s">
+        <v>231</v>
+      </c>
+      <c r="J34" t="s">
+        <v>232</v>
+      </c>
+      <c r="K34" t="s">
         <v>233</v>
-      </c>
-      <c r="B34" t="s">
-        <v>234</v>
-      </c>
-      <c r="C34" t="s">
-        <v>235</v>
-      </c>
-      <c r="D34" t="s">
-        <v>236</v>
-      </c>
-      <c r="E34" t="s">
-        <v>237</v>
-      </c>
-      <c r="J34" t="s">
-        <v>238</v>
-      </c>
-      <c r="K34" t="s">
-        <v>239</v>
       </c>
       <c r="L34">
         <v>15</v>
@@ -3495,30 +3519,30 @@
         <v>0</v>
       </c>
       <c r="Q34" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B35" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C35" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D35" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E35" t="s">
         <v>22</v>
       </c>
       <c r="J35" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="K35" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="L35">
         <v>0</v>
@@ -3536,30 +3560,30 @@
         <v>0</v>
       </c>
       <c r="Q35" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B36" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="C36" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="D36" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E36" t="s">
         <v>19</v>
       </c>
       <c r="J36" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="K36" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="L36">
         <v>0</v>
@@ -3577,30 +3601,30 @@
         <v>46</v>
       </c>
       <c r="Q36" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" t="s">
-        <v>254</v>
+        <v>440</v>
       </c>
       <c r="B37" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C37" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D37" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="E37" t="s">
         <v>112</v>
       </c>
       <c r="J37" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="K37" s="15" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="L37">
         <v>0</v>
@@ -3618,30 +3642,30 @@
         <v>0</v>
       </c>
       <c r="Q37" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B38" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C38" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D38" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="E38" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="J38" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="K38" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="L38">
         <v>0</v>
@@ -3659,18 +3683,18 @@
         <v>0</v>
       </c>
       <c r="Q38" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="B39" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="C39" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D39" t="s">
         <v>77</v>
@@ -3679,10 +3703,10 @@
         <v>22</v>
       </c>
       <c r="J39" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="K39" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="L39">
         <v>0</v>
@@ -3700,30 +3724,30 @@
         <v>0</v>
       </c>
       <c r="Q39" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" t="s">
-        <v>273</v>
+        <v>441</v>
       </c>
       <c r="B40" s="10">
         <v>13204</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="J40" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="L40">
         <v>0</v>
@@ -3741,27 +3765,27 @@
         <v>0</v>
       </c>
       <c r="Q40" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:17">
       <c r="A41" t="s">
-        <v>278</v>
+        <v>442</v>
       </c>
       <c r="B41" s="10">
         <v>17976</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>39</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K41" s="15" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="L41">
         <v>1</v>
@@ -3781,13 +3805,13 @@
     </row>
     <row r="42" spans="1:17">
       <c r="A42" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="B42" s="10">
         <v>23238</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>39</v>
@@ -3796,10 +3820,10 @@
         <v>19</v>
       </c>
       <c r="J42" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="K42" s="15" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -3819,13 +3843,13 @@
     </row>
     <row r="43" spans="1:17">
       <c r="A43" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="B43" s="11">
         <v>22119</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>39</v>
@@ -3843,10 +3867,10 @@
         <v>19</v>
       </c>
       <c r="J43" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>438</v>
+        <v>429</v>
       </c>
       <c r="L43">
         <v>84</v>
@@ -3888,28 +3912,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3920,22 +3944,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D2" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="E2" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="F2" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="G2" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="H2" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3946,19 +3970,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="E3" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="F3" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="G3" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="H3" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3969,22 +3993,22 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
+        <v>286</v>
+      </c>
+      <c r="D4" t="s">
         <v>295</v>
       </c>
-      <c r="D4" t="s">
-        <v>304</v>
-      </c>
       <c r="E4" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
       <c r="F4" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="G4" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="H4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -3995,22 +4019,22 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D5" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="E5" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="F5" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="G5" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="H5" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -4021,19 +4045,19 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="E6" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="F6" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="G6" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="H6" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -4044,22 +4068,22 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D7" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="E7" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
       <c r="F7" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="G7" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="H7" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -4070,13 +4094,13 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G8" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="H8" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -4087,13 +4111,13 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G9" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="H9" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -4104,13 +4128,13 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G10" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H10" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -4121,22 +4145,22 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D11" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="E11" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="F11" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="G11" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="H11" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -4147,22 +4171,22 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D12" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="E12" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="F12" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="G12" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="H12" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -4173,13 +4197,13 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G13" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="H13" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -4190,13 +4214,13 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G14" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="H14" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4207,22 +4231,22 @@
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D15" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="E15" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="F15" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="G15" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="H15" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -4233,22 +4257,22 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D16" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="E16" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="F16" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="G16" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="H16" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -4259,13 +4283,13 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G17" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="H17" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -4276,13 +4300,13 @@
         <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G18" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="H18" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -4293,22 +4317,22 @@
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D19" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="E19" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="F19" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="G19" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="H19" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -4319,22 +4343,22 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D20" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="E20" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="F20" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="G20" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="H20" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -4345,13 +4369,13 @@
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G21" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="H21" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -4362,13 +4386,13 @@
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G22" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="H22" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -4379,13 +4403,13 @@
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G23" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="H23" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -4396,22 +4420,22 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D24" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="E24" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="F24" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="G24" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="H24" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -4422,22 +4446,22 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D25" t="s">
-        <v>349</v>
+        <v>340</v>
       </c>
       <c r="E25" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="F25" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="G25" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="H25" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -4448,13 +4472,13 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G26" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H26" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -4465,13 +4489,13 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G27" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H27" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -4482,13 +4506,13 @@
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G28" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H28" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -4499,22 +4523,22 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D29" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="E29" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="F29" t="s">
-        <v>355</v>
+        <v>346</v>
       </c>
       <c r="G29" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="H29" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -4525,22 +4549,22 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D30" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="E30" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="F30" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="G30" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="H30" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -4551,13 +4575,13 @@
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G31" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="H31" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -4568,13 +4592,13 @@
         <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G32" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H32" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -4585,13 +4609,13 @@
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G33" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H33" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -4602,22 +4626,22 @@
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D34" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="E34" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="F34" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
       <c r="G34" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="H34" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -4628,22 +4652,22 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D35" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="E35" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="F35" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="G35" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="H35" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -4654,13 +4678,13 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G36" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="H36" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -4671,13 +4695,13 @@
         <v>3</v>
       </c>
       <c r="C37" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G37" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H37" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -4688,13 +4712,13 @@
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G38" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H38" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -4705,22 +4729,22 @@
         <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D39" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="E39" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="F39" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="G39" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="H39" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -4731,22 +4755,22 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D40" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="E40" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="F40" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="G40" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="H40" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -4757,13 +4781,13 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G41" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="H41" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -4774,13 +4798,13 @@
         <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G42" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H42" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -4791,13 +4815,13 @@
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G43" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H43" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -4808,22 +4832,22 @@
         <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D44" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="E44" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="F44" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="G44" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="H44" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -4834,22 +4858,22 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D45" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="E45" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="F45" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="G45" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="H45" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -4860,13 +4884,13 @@
         <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G46" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H46" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -4877,13 +4901,13 @@
         <v>3</v>
       </c>
       <c r="C47" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G47" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H47" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -4894,13 +4918,13 @@
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G48" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="H48" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -4911,22 +4935,22 @@
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D49" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="E49" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="F49" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="G49" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="H49" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -4937,22 +4961,22 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D50" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="E50" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="F50" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="G50" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="H50" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -4963,13 +4987,13 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G51" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H51" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -4980,13 +5004,13 @@
         <v>3</v>
       </c>
       <c r="C52" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G52" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H52" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -4997,13 +5021,13 @@
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G53" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="H53" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -5014,22 +5038,22 @@
         <v>5</v>
       </c>
       <c r="C54" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D54" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="E54" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="F54" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="G54" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="H54" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -5040,22 +5064,22 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D55" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="E55" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="F55" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="G55" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="H55" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -5066,22 +5090,22 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D56" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="E56" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="F56" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="G56" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="H56" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -5092,13 +5116,13 @@
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G57" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H57" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -5109,13 +5133,13 @@
         <v>3</v>
       </c>
       <c r="C58" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G58" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="H58" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -5126,13 +5150,13 @@
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G59" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="H59" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -5143,22 +5167,22 @@
         <v>5</v>
       </c>
       <c r="C60" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D60" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="E60" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="F60" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
       <c r="G60" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="H60" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -5169,22 +5193,22 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D61" t="s">
+        <v>386</v>
+      </c>
+      <c r="E61" t="s">
+        <v>387</v>
+      </c>
+      <c r="F61" t="s">
+        <v>394</v>
+      </c>
+      <c r="G61" t="s">
         <v>395</v>
       </c>
-      <c r="E61" t="s">
-        <v>396</v>
-      </c>
-      <c r="F61" t="s">
-        <v>403</v>
-      </c>
-      <c r="G61" t="s">
-        <v>404</v>
-      </c>
       <c r="H61" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -5195,13 +5219,13 @@
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G62" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="H62" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -5212,13 +5236,13 @@
         <v>3</v>
       </c>
       <c r="C63" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G63" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="H63" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -5229,13 +5253,13 @@
         <v>4</v>
       </c>
       <c r="C64" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G64" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="H64" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -5246,22 +5270,22 @@
         <v>5</v>
       </c>
       <c r="C65" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D65" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="E65" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="F65" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="G65" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="H65" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -5272,22 +5296,22 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D66" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="E66" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="F66" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="G66" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="H66" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -5298,13 +5322,13 @@
         <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G67" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="H67" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -5315,13 +5339,13 @@
         <v>3</v>
       </c>
       <c r="C68" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G68" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="H68" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -5332,13 +5356,13 @@
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G69" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="H69" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -5349,36 +5373,36 @@
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="E70" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
       <c r="F70" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="G70" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="H70" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B71">
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="G71" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="H71" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Data] Schema and xlsx files update
</commit_message>
<xml_diff>
--- a/server/coach-infos.xlsx
+++ b/server/coach-infos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\samir\archifoot\server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3BA431E-21FB-4D26-9B2A-35DD09D9DE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470699DE-78B9-48D2-AD18-4ADA1092D4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="448">
   <si>
     <t>nom_complet</t>
   </si>
@@ -916,18 +916,12 @@
     <t xml:space="preserve">Cheraga </t>
   </si>
   <si>
-    <t xml:space="preserve">MAAOUCHE Mohamed </t>
-  </si>
-  <si>
     <t xml:space="preserve">El Biar </t>
   </si>
   <si>
     <t>1953/1975</t>
   </si>
   <si>
-    <t xml:space="preserve">Menad Djamel </t>
-  </si>
-  <si>
     <t>El Biar</t>
   </si>
   <si>
@@ -1430,6 +1424,27 @@
   </si>
   <si>
     <t xml:space="preserve">Rachid Cherradi </t>
+  </si>
+  <si>
+    <t>18/04/1931</t>
+  </si>
+  <si>
+    <t>24/02/1936</t>
+  </si>
+  <si>
+    <t>19/03/1949</t>
+  </si>
+  <si>
+    <t>15/08/1963</t>
+  </si>
+  <si>
+    <t>22/07/1960</t>
+  </si>
+  <si>
+    <t>Maouche Mohamed</t>
+  </si>
+  <si>
+    <t>Menad Djamel</t>
   </si>
 </sst>
 </file>
@@ -1552,7 +1567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1567,12 +1582,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1582,11 +1591,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -1608,7 +1628,7 @@
   <autoFilter ref="A1:Q43" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="nom_complet"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="date_naissance"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="date_naissance" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ville_naissance"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="region_naissance"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="pays_naissance"/>
@@ -1621,7 +1641,7 @@
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="nombre_selections_joueur"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="nombre_selections_joueur_equipe_étrangère"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="nombre_matches_entraineur_national"/>
-    <tableColumn id="3" xr3:uid="{47C92A9E-293B-4B4A-AD95-1DB2C6D4CB4B}" name="Nombre de fois solicités" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{47C92A9E-293B-4B4A-AD95-1DB2C6D4CB4B}" name="Nombre de fois solicités" dataDxfId="1"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="nombre_matches_co_entraineur_/assitants"/>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="description"/>
   </tableColumns>
@@ -1979,8 +1999,8 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="13" t="s">
-        <v>277</v>
+      <c r="O1" s="11" t="s">
+        <v>275</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>14</v>
@@ -1993,7 +2013,7 @@
       <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="15" t="s">
         <v>17</v>
       </c>
       <c r="C2" t="s">
@@ -2014,10 +2034,10 @@
       <c r="I2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="15" t="s">
-        <v>430</v>
-      </c>
-      <c r="K2" s="15" t="s">
+      <c r="J2" s="13" t="s">
+        <v>428</v>
+      </c>
+      <c r="K2" s="13" t="s">
         <v>21</v>
       </c>
       <c r="L2">
@@ -2029,7 +2049,7 @@
       <c r="N2">
         <v>2</v>
       </c>
-      <c r="O2" s="14">
+      <c r="O2" s="12">
         <v>1</v>
       </c>
       <c r="P2">
@@ -2043,7 +2063,7 @@
       <c r="A3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C3" t="s">
@@ -2079,7 +2099,7 @@
       <c r="N3">
         <v>1</v>
       </c>
-      <c r="O3" s="14">
+      <c r="O3" s="12">
         <v>1</v>
       </c>
       <c r="P3">
@@ -2093,7 +2113,7 @@
       <c r="A4" t="s">
         <v>33</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="15" t="s">
         <v>34</v>
       </c>
       <c r="C4" t="s">
@@ -2117,11 +2137,11 @@
       <c r="I4" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="15" t="s">
-        <v>431</v>
+      <c r="J4" s="13" t="s">
+        <v>429</v>
       </c>
       <c r="K4" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -2132,7 +2152,7 @@
       <c r="N4">
         <v>7</v>
       </c>
-      <c r="O4" s="14">
+      <c r="O4" s="12">
         <v>4</v>
       </c>
       <c r="P4">
@@ -2146,7 +2166,7 @@
       <c r="A5" t="s">
         <v>41</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="15" t="s">
         <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -2167,8 +2187,8 @@
       <c r="I5" t="s">
         <v>39</v>
       </c>
-      <c r="J5" s="15" t="s">
-        <v>432</v>
+      <c r="J5" s="13" t="s">
+        <v>430</v>
       </c>
       <c r="K5" t="s">
         <v>44</v>
@@ -2182,7 +2202,7 @@
       <c r="N5">
         <v>13</v>
       </c>
-      <c r="O5" s="14">
+      <c r="O5" s="12">
         <v>3</v>
       </c>
       <c r="P5">
@@ -2196,7 +2216,7 @@
       <c r="A6" t="s">
         <v>46</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="15" t="s">
         <v>47</v>
       </c>
       <c r="C6" t="s">
@@ -2220,11 +2240,11 @@
       <c r="I6" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="15" t="s">
-        <v>433</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>411</v>
+      <c r="J6" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>409</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -2235,7 +2255,7 @@
       <c r="N6">
         <v>0</v>
       </c>
-      <c r="O6" s="14">
+      <c r="O6" s="12">
         <v>2</v>
       </c>
       <c r="P6">
@@ -2249,7 +2269,7 @@
       <c r="A7" t="s">
         <v>53</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="15" t="s">
         <v>54</v>
       </c>
       <c r="C7" t="s">
@@ -2285,7 +2305,7 @@
       <c r="N7">
         <v>25</v>
       </c>
-      <c r="O7" s="14">
+      <c r="O7" s="12">
         <v>1</v>
       </c>
       <c r="P7">
@@ -2299,7 +2319,7 @@
       <c r="A8" t="s">
         <v>62</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="15" t="s">
         <v>63</v>
       </c>
       <c r="C8" t="s">
@@ -2323,8 +2343,8 @@
       <c r="J8" t="s">
         <v>64</v>
       </c>
-      <c r="K8" s="15" t="s">
-        <v>412</v>
+      <c r="K8" s="13" t="s">
+        <v>410</v>
       </c>
       <c r="L8">
         <v>10</v>
@@ -2335,7 +2355,7 @@
       <c r="N8">
         <v>11</v>
       </c>
-      <c r="O8" s="14">
+      <c r="O8" s="12">
         <v>2</v>
       </c>
       <c r="P8">
@@ -2349,7 +2369,7 @@
       <c r="A9" t="s">
         <v>66</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="15" t="s">
         <v>67</v>
       </c>
       <c r="C9" t="s">
@@ -2373,8 +2393,8 @@
       <c r="J9" t="s">
         <v>71</v>
       </c>
-      <c r="K9" s="15" t="s">
-        <v>413</v>
+      <c r="K9" s="13" t="s">
+        <v>411</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -2385,7 +2405,7 @@
       <c r="N9">
         <v>26</v>
       </c>
-      <c r="O9" s="14">
+      <c r="O9" s="12">
         <v>5</v>
       </c>
       <c r="P9">
@@ -2399,7 +2419,7 @@
       <c r="A10" t="s">
         <v>73</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="15" t="s">
         <v>74</v>
       </c>
       <c r="C10" t="s">
@@ -2438,7 +2458,7 @@
       <c r="N10">
         <v>59</v>
       </c>
-      <c r="O10" s="14">
+      <c r="O10" s="12">
         <v>2</v>
       </c>
       <c r="P10">
@@ -2452,7 +2472,7 @@
       <c r="A11" t="s">
         <v>81</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="15" t="s">
         <v>82</v>
       </c>
       <c r="C11" t="s">
@@ -2467,8 +2487,8 @@
       <c r="J11" t="s">
         <v>84</v>
       </c>
-      <c r="K11" s="15" t="s">
-        <v>414</v>
+      <c r="K11" s="13" t="s">
+        <v>412</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -2479,7 +2499,7 @@
       <c r="N11">
         <v>0</v>
       </c>
-      <c r="O11" s="14">
+      <c r="O11" s="12">
         <v>1</v>
       </c>
       <c r="P11">
@@ -2493,7 +2513,7 @@
       <c r="A12" t="s">
         <v>86</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="15" t="s">
         <v>87</v>
       </c>
       <c r="C12" t="s">
@@ -2523,7 +2543,7 @@
       <c r="N12">
         <v>0</v>
       </c>
-      <c r="O12" s="14">
+      <c r="O12" s="12">
         <v>1</v>
       </c>
       <c r="P12">
@@ -2535,10 +2555,10 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" t="s">
-        <v>410</v>
-      </c>
-      <c r="B13" s="5">
-        <v>11441</v>
+        <v>408</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>441</v>
       </c>
       <c r="C13" t="s">
         <v>93</v>
@@ -2561,8 +2581,8 @@
       <c r="J13" t="s">
         <v>97</v>
       </c>
-      <c r="K13" s="15" t="s">
-        <v>415</v>
+      <c r="K13" s="13" t="s">
+        <v>413</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -2573,7 +2593,7 @@
       <c r="N13">
         <v>12</v>
       </c>
-      <c r="O13" s="14">
+      <c r="O13" s="12">
         <v>1</v>
       </c>
       <c r="P13">
@@ -2587,7 +2607,7 @@
       <c r="A14" t="s">
         <v>99</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="15" t="s">
         <v>100</v>
       </c>
       <c r="C14" t="s">
@@ -2623,7 +2643,7 @@
       <c r="N14">
         <v>21</v>
       </c>
-      <c r="O14" s="14">
+      <c r="O14" s="12">
         <v>2</v>
       </c>
       <c r="P14">
@@ -2637,7 +2657,7 @@
       <c r="A15" t="s">
         <v>108</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="15" t="s">
         <v>109</v>
       </c>
       <c r="C15" t="s">
@@ -2673,7 +2693,7 @@
       <c r="N15">
         <v>8</v>
       </c>
-      <c r="O15" s="14">
+      <c r="O15" s="12">
         <v>3</v>
       </c>
       <c r="P15">
@@ -2687,7 +2707,7 @@
       <c r="A16" t="s">
         <v>119</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="15" t="s">
         <v>120</v>
       </c>
       <c r="C16" t="s">
@@ -2723,7 +2743,7 @@
       <c r="N16">
         <v>1</v>
       </c>
-      <c r="O16" s="14">
+      <c r="O16" s="12">
         <v>1</v>
       </c>
       <c r="P16">
@@ -2737,7 +2757,7 @@
       <c r="A17" t="s">
         <v>128</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="15" t="s">
         <v>129</v>
       </c>
       <c r="C17" t="s">
@@ -2773,7 +2793,7 @@
       <c r="N17">
         <v>21</v>
       </c>
-      <c r="O17" s="14">
+      <c r="O17" s="12">
         <v>2</v>
       </c>
       <c r="P17">
@@ -2787,7 +2807,7 @@
       <c r="A18" t="s">
         <v>138</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="15" t="s">
         <v>139</v>
       </c>
       <c r="C18" t="s">
@@ -2802,8 +2822,8 @@
       <c r="J18" t="s">
         <v>141</v>
       </c>
-      <c r="K18" s="15" t="s">
-        <v>416</v>
+      <c r="K18" s="13" t="s">
+        <v>414</v>
       </c>
       <c r="L18">
         <v>2</v>
@@ -2814,7 +2834,7 @@
       <c r="N18">
         <v>72</v>
       </c>
-      <c r="O18" s="14">
+      <c r="O18" s="12">
         <v>6</v>
       </c>
       <c r="P18">
@@ -2828,7 +2848,7 @@
       <c r="A19" t="s">
         <v>143</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="15" t="s">
         <v>144</v>
       </c>
       <c r="C19" t="s">
@@ -2852,8 +2872,8 @@
       <c r="J19" t="s">
         <v>149</v>
       </c>
-      <c r="K19" s="15" t="s">
-        <v>417</v>
+      <c r="K19" s="13" t="s">
+        <v>415</v>
       </c>
       <c r="L19">
         <v>10</v>
@@ -2864,7 +2884,7 @@
       <c r="N19">
         <v>18</v>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="12">
         <v>1</v>
       </c>
       <c r="P19">
@@ -2878,7 +2898,7 @@
       <c r="A20" t="s">
         <v>151</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="15" t="s">
         <v>152</v>
       </c>
       <c r="C20" t="s">
@@ -2902,8 +2922,8 @@
       <c r="J20" t="s">
         <v>156</v>
       </c>
-      <c r="K20" s="15" t="s">
-        <v>418</v>
+      <c r="K20" s="13" t="s">
+        <v>416</v>
       </c>
       <c r="L20">
         <v>1</v>
@@ -2914,7 +2934,7 @@
       <c r="N20">
         <v>24</v>
       </c>
-      <c r="O20" s="14">
+      <c r="O20" s="12">
         <v>2</v>
       </c>
       <c r="P20">
@@ -2925,10 +2945,10 @@
       </c>
     </row>
     <row r="21" spans="1:17" ht="15.75">
-      <c r="A21" s="16" t="s">
-        <v>434</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="A21" s="14" t="s">
+        <v>432</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>158</v>
       </c>
       <c r="C21" t="s">
@@ -2955,7 +2975,7 @@
       <c r="N21">
         <v>20</v>
       </c>
-      <c r="O21" s="14">
+      <c r="O21" s="12">
         <v>3</v>
       </c>
       <c r="P21">
@@ -2967,9 +2987,9 @@
     </row>
     <row r="22" spans="1:17">
       <c r="A22" t="s">
-        <v>435</v>
-      </c>
-      <c r="B22" t="s">
+        <v>433</v>
+      </c>
+      <c r="B22" s="15" t="s">
         <v>162</v>
       </c>
       <c r="C22" s="2" t="s">
@@ -3005,7 +3025,7 @@
       <c r="N22">
         <v>17</v>
       </c>
-      <c r="O22" s="14">
+      <c r="O22" s="12">
         <v>2</v>
       </c>
       <c r="P22">
@@ -3019,7 +3039,7 @@
       <c r="A23" t="s">
         <v>166</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="15" t="s">
         <v>167</v>
       </c>
       <c r="C23" s="2" t="s">
@@ -3034,8 +3054,8 @@
       <c r="J23" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="K23" s="15" t="s">
-        <v>419</v>
+      <c r="K23" s="13" t="s">
+        <v>417</v>
       </c>
       <c r="L23">
         <v>90</v>
@@ -3046,7 +3066,7 @@
       <c r="N23">
         <v>25</v>
       </c>
-      <c r="O23" s="14">
+      <c r="O23" s="12">
         <v>3</v>
       </c>
       <c r="P23">
@@ -3060,7 +3080,7 @@
       <c r="A24" t="s">
         <v>170</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="15" t="s">
         <v>171</v>
       </c>
       <c r="C24" t="s">
@@ -3075,8 +3095,8 @@
       <c r="J24" t="s">
         <v>174</v>
       </c>
-      <c r="K24" s="15" t="s">
-        <v>420</v>
+      <c r="K24" s="13" t="s">
+        <v>418</v>
       </c>
       <c r="L24">
         <v>73</v>
@@ -3087,7 +3107,7 @@
       <c r="N24">
         <v>7</v>
       </c>
-      <c r="O24" s="14">
+      <c r="O24" s="12">
         <v>2</v>
       </c>
       <c r="P24">
@@ -3101,7 +3121,7 @@
       <c r="A25" t="s">
         <v>176</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="15" t="s">
         <v>177</v>
       </c>
       <c r="C25" t="s">
@@ -3134,7 +3154,7 @@
       <c r="N25">
         <v>0</v>
       </c>
-      <c r="O25" s="14">
+      <c r="O25" s="12">
         <v>1</v>
       </c>
       <c r="P25">
@@ -3148,7 +3168,7 @@
       <c r="A26" t="s">
         <v>182</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="15" t="s">
         <v>183</v>
       </c>
       <c r="C26" t="s">
@@ -3163,8 +3183,8 @@
       <c r="J26" t="s">
         <v>186</v>
       </c>
-      <c r="K26" s="15" t="s">
-        <v>421</v>
+      <c r="K26" s="13" t="s">
+        <v>419</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -3175,7 +3195,7 @@
       <c r="N26">
         <v>0</v>
       </c>
-      <c r="O26" s="14">
+      <c r="O26" s="12">
         <v>1</v>
       </c>
       <c r="P26">
@@ -3189,7 +3209,7 @@
       <c r="A27" t="s">
         <v>188</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="15" t="s">
         <v>189</v>
       </c>
       <c r="C27" t="s">
@@ -3204,8 +3224,8 @@
       <c r="J27" t="s">
         <v>191</v>
       </c>
-      <c r="K27" s="15" t="s">
-        <v>422</v>
+      <c r="K27" s="13" t="s">
+        <v>420</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -3216,7 +3236,7 @@
       <c r="N27">
         <v>7</v>
       </c>
-      <c r="O27" s="14">
+      <c r="O27" s="12">
         <v>1</v>
       </c>
       <c r="P27">
@@ -3230,7 +3250,7 @@
       <c r="A28" t="s">
         <v>193</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="15" t="s">
         <v>194</v>
       </c>
       <c r="C28" t="s">
@@ -3245,8 +3265,8 @@
       <c r="J28" t="s">
         <v>197</v>
       </c>
-      <c r="K28" s="15" t="s">
-        <v>423</v>
+      <c r="K28" s="13" t="s">
+        <v>421</v>
       </c>
       <c r="L28">
         <v>3</v>
@@ -3257,7 +3277,7 @@
       <c r="N28">
         <v>5</v>
       </c>
-      <c r="O28" s="14">
+      <c r="O28" s="12">
         <v>1</v>
       </c>
       <c r="P28">
@@ -3269,9 +3289,9 @@
     </row>
     <row r="29" spans="1:17">
       <c r="A29" t="s">
-        <v>436</v>
-      </c>
-      <c r="B29" t="s">
+        <v>434</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>199</v>
       </c>
       <c r="C29" t="s">
@@ -3286,8 +3306,8 @@
       <c r="J29" t="s">
         <v>200</v>
       </c>
-      <c r="K29" s="15" t="s">
-        <v>421</v>
+      <c r="K29" s="13" t="s">
+        <v>419</v>
       </c>
       <c r="L29">
         <v>0</v>
@@ -3298,7 +3318,7 @@
       <c r="N29">
         <v>0</v>
       </c>
-      <c r="O29" s="14">
+      <c r="O29" s="12">
         <v>1</v>
       </c>
       <c r="P29">
@@ -3312,7 +3332,7 @@
       <c r="A30" t="s">
         <v>202</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="15" t="s">
         <v>203</v>
       </c>
       <c r="C30" t="s">
@@ -3339,7 +3359,7 @@
       <c r="N30">
         <v>11</v>
       </c>
-      <c r="O30" s="14">
+      <c r="O30" s="12">
         <v>2</v>
       </c>
       <c r="P30">
@@ -3351,9 +3371,9 @@
     </row>
     <row r="31" spans="1:17">
       <c r="A31" t="s">
-        <v>437</v>
-      </c>
-      <c r="B31" t="s">
+        <v>435</v>
+      </c>
+      <c r="B31" s="15" t="s">
         <v>210</v>
       </c>
       <c r="C31" t="s">
@@ -3389,7 +3409,7 @@
       <c r="N31">
         <v>6</v>
       </c>
-      <c r="O31" s="14">
+      <c r="O31" s="12">
         <v>1</v>
       </c>
       <c r="P31">
@@ -3403,7 +3423,7 @@
       <c r="A32" t="s">
         <v>218</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="15" t="s">
         <v>219</v>
       </c>
       <c r="C32" t="s">
@@ -3430,7 +3450,7 @@
       <c r="N32">
         <v>12</v>
       </c>
-      <c r="O32" s="14">
+      <c r="O32" s="12">
         <v>1</v>
       </c>
       <c r="P32">
@@ -3442,9 +3462,9 @@
     </row>
     <row r="33" spans="1:17">
       <c r="A33" t="s">
-        <v>438</v>
-      </c>
-      <c r="B33" t="s">
+        <v>436</v>
+      </c>
+      <c r="B33" s="15" t="s">
         <v>225</v>
       </c>
       <c r="C33" t="s">
@@ -3459,8 +3479,8 @@
       <c r="J33" t="s">
         <v>226</v>
       </c>
-      <c r="K33" s="15" t="s">
-        <v>424</v>
+      <c r="K33" s="13" t="s">
+        <v>422</v>
       </c>
       <c r="L33">
         <v>0</v>
@@ -3471,7 +3491,7 @@
       <c r="N33">
         <v>4</v>
       </c>
-      <c r="O33" s="14">
+      <c r="O33" s="12">
         <v>1</v>
       </c>
       <c r="P33">
@@ -3483,9 +3503,9 @@
     </row>
     <row r="34" spans="1:17">
       <c r="A34" t="s">
-        <v>439</v>
-      </c>
-      <c r="B34" t="s">
+        <v>437</v>
+      </c>
+      <c r="B34" s="15" t="s">
         <v>228</v>
       </c>
       <c r="C34" t="s">
@@ -3512,7 +3532,7 @@
       <c r="N34">
         <v>35</v>
       </c>
-      <c r="O34" s="14">
+      <c r="O34" s="12">
         <v>1</v>
       </c>
       <c r="P34">
@@ -3526,7 +3546,7 @@
       <c r="A35" t="s">
         <v>235</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="15" t="s">
         <v>236</v>
       </c>
       <c r="C35" t="s">
@@ -3553,7 +3573,7 @@
       <c r="N35">
         <v>21</v>
       </c>
-      <c r="O35" s="14">
+      <c r="O35" s="12">
         <v>1</v>
       </c>
       <c r="P35">
@@ -3567,7 +3587,7 @@
       <c r="A36" t="s">
         <v>242</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="15" t="s">
         <v>243</v>
       </c>
       <c r="C36" t="s">
@@ -3594,7 +3614,7 @@
       <c r="N36">
         <v>1</v>
       </c>
-      <c r="O36" s="14">
+      <c r="O36" s="12">
         <v>1</v>
       </c>
       <c r="P36">
@@ -3606,9 +3626,9 @@
     </row>
     <row r="37" spans="1:17">
       <c r="A37" t="s">
-        <v>440</v>
-      </c>
-      <c r="B37" t="s">
+        <v>438</v>
+      </c>
+      <c r="B37" s="15" t="s">
         <v>248</v>
       </c>
       <c r="C37" t="s">
@@ -3623,8 +3643,8 @@
       <c r="J37" t="s">
         <v>251</v>
       </c>
-      <c r="K37" s="15" t="s">
-        <v>425</v>
+      <c r="K37" s="13" t="s">
+        <v>423</v>
       </c>
       <c r="L37">
         <v>0</v>
@@ -3635,7 +3655,7 @@
       <c r="N37">
         <v>2</v>
       </c>
-      <c r="O37" s="14">
+      <c r="O37" s="12">
         <v>1</v>
       </c>
       <c r="P37">
@@ -3649,7 +3669,7 @@
       <c r="A38" t="s">
         <v>253</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="15" t="s">
         <v>254</v>
       </c>
       <c r="C38" t="s">
@@ -3676,7 +3696,7 @@
       <c r="N38">
         <v>5</v>
       </c>
-      <c r="O38" s="14">
+      <c r="O38" s="12">
         <v>1</v>
       </c>
       <c r="P38">
@@ -3690,7 +3710,7 @@
       <c r="A39" t="s">
         <v>261</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C39" t="s">
@@ -3717,7 +3737,7 @@
       <c r="N39">
         <v>64</v>
       </c>
-      <c r="O39" s="14">
+      <c r="O39" s="12">
         <v>1</v>
       </c>
       <c r="P39">
@@ -3729,10 +3749,10 @@
     </row>
     <row r="40" spans="1:17">
       <c r="A40" t="s">
-        <v>441</v>
-      </c>
-      <c r="B40" s="10">
-        <v>13204</v>
+        <v>439</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>442</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>266</v>
@@ -3746,8 +3766,8 @@
       <c r="J40" t="s">
         <v>268</v>
       </c>
-      <c r="K40" s="15" t="s">
-        <v>426</v>
+      <c r="K40" s="13" t="s">
+        <v>424</v>
       </c>
       <c r="L40">
         <v>0</v>
@@ -3758,7 +3778,7 @@
       <c r="N40">
         <v>25</v>
       </c>
-      <c r="O40" s="14">
+      <c r="O40" s="12">
         <v>1</v>
       </c>
       <c r="P40">
@@ -3770,10 +3790,10 @@
     </row>
     <row r="41" spans="1:17">
       <c r="A41" t="s">
-        <v>442</v>
-      </c>
-      <c r="B41" s="10">
-        <v>17976</v>
+        <v>440</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>443</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>270</v>
@@ -3784,8 +3804,8 @@
       <c r="E41" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="K41" s="15" t="s">
-        <v>427</v>
+      <c r="K41" s="13" t="s">
+        <v>425</v>
       </c>
       <c r="L41">
         <v>1</v>
@@ -3796,7 +3816,7 @@
       <c r="N41">
         <v>1</v>
       </c>
-      <c r="O41" s="14">
+      <c r="O41" s="12">
         <v>1</v>
       </c>
       <c r="P41">
@@ -3804,14 +3824,14 @@
       </c>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" t="s">
+      <c r="A42" s="13" t="s">
+        <v>446</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>444</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>271</v>
-      </c>
-      <c r="B42" s="10">
-        <v>23238</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>272</v>
       </c>
       <c r="D42" s="7" t="s">
         <v>39</v>
@@ -3820,10 +3840,10 @@
         <v>19</v>
       </c>
       <c r="J42" t="s">
-        <v>273</v>
-      </c>
-      <c r="K42" s="15" t="s">
-        <v>428</v>
+        <v>272</v>
+      </c>
+      <c r="K42" s="13" t="s">
+        <v>426</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -3834,7 +3854,7 @@
       <c r="N42">
         <v>0</v>
       </c>
-      <c r="O42" s="14">
+      <c r="O42" s="12">
         <v>1</v>
       </c>
       <c r="P42">
@@ -3842,14 +3862,14 @@
       </c>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" t="s">
-        <v>274</v>
-      </c>
-      <c r="B43" s="11">
-        <v>22119</v>
+      <c r="A43" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>445</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D43" s="7" t="s">
         <v>39</v>
@@ -3857,7 +3877,7 @@
       <c r="E43" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="F43" s="12">
+      <c r="F43" s="10">
         <v>45738</v>
       </c>
       <c r="G43" t="s">
@@ -3867,10 +3887,10 @@
         <v>19</v>
       </c>
       <c r="J43" t="s">
-        <v>276</v>
-      </c>
-      <c r="K43" s="15" t="s">
-        <v>429</v>
+        <v>274</v>
+      </c>
+      <c r="K43" s="13" t="s">
+        <v>427</v>
       </c>
       <c r="L43">
         <v>84</v>
@@ -3881,7 +3901,7 @@
       <c r="N43">
         <v>0</v>
       </c>
-      <c r="O43" s="14">
+      <c r="O43" s="12">
         <v>1</v>
       </c>
       <c r="P43">
@@ -3912,28 +3932,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3944,22 +3964,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E2" t="s">
         <v>286</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>287</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>288</v>
       </c>
-      <c r="F2" t="s">
-        <v>289</v>
-      </c>
-      <c r="G2" t="s">
-        <v>290</v>
-      </c>
       <c r="H2" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -3970,19 +3990,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E3" t="s">
+        <v>290</v>
+      </c>
+      <c r="F3" t="s">
+        <v>291</v>
+      </c>
+      <c r="G3" t="s">
         <v>292</v>
       </c>
-      <c r="F3" t="s">
-        <v>293</v>
-      </c>
-      <c r="G3" t="s">
-        <v>294</v>
-      </c>
       <c r="H3" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -3993,22 +4013,22 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D4" t="s">
+        <v>293</v>
+      </c>
+      <c r="E4" t="s">
+        <v>294</v>
+      </c>
+      <c r="F4" t="s">
         <v>295</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>296</v>
       </c>
-      <c r="F4" t="s">
-        <v>297</v>
-      </c>
-      <c r="G4" t="s">
-        <v>298</v>
-      </c>
       <c r="H4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -4019,22 +4039,22 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D5" t="s">
+        <v>285</v>
+      </c>
+      <c r="E5" t="s">
         <v>286</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>287</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>288</v>
       </c>
-      <c r="F5" t="s">
-        <v>289</v>
-      </c>
-      <c r="G5" t="s">
-        <v>290</v>
-      </c>
       <c r="H5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -4045,19 +4065,19 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E6" t="s">
+        <v>290</v>
+      </c>
+      <c r="F6" t="s">
+        <v>291</v>
+      </c>
+      <c r="G6" t="s">
         <v>292</v>
       </c>
-      <c r="F6" t="s">
-        <v>293</v>
-      </c>
-      <c r="G6" t="s">
-        <v>294</v>
-      </c>
       <c r="H6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -4068,22 +4088,22 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D7" t="s">
+        <v>297</v>
+      </c>
+      <c r="E7" t="s">
+        <v>298</v>
+      </c>
+      <c r="F7" t="s">
         <v>299</v>
       </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>300</v>
       </c>
-      <c r="F7" t="s">
-        <v>301</v>
-      </c>
-      <c r="G7" t="s">
-        <v>302</v>
-      </c>
       <c r="H7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -4094,13 +4114,13 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G8" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H8" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -4111,13 +4131,13 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
+        <v>301</v>
+      </c>
+      <c r="G9" t="s">
         <v>303</v>
       </c>
-      <c r="G9" t="s">
-        <v>305</v>
-      </c>
       <c r="H9" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -4128,13 +4148,13 @@
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G10" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H10" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -4145,22 +4165,22 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D11" t="s">
+        <v>305</v>
+      </c>
+      <c r="E11" t="s">
+        <v>306</v>
+      </c>
+      <c r="F11" t="s">
         <v>307</v>
       </c>
-      <c r="E11" t="s">
+      <c r="G11" t="s">
         <v>308</v>
       </c>
-      <c r="F11" t="s">
-        <v>309</v>
-      </c>
-      <c r="G11" t="s">
-        <v>310</v>
-      </c>
       <c r="H11" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -4171,22 +4191,22 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D12" t="s">
+        <v>309</v>
+      </c>
+      <c r="E12" t="s">
+        <v>310</v>
+      </c>
+      <c r="F12" t="s">
         <v>311</v>
       </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
         <v>312</v>
       </c>
-      <c r="F12" t="s">
-        <v>313</v>
-      </c>
-      <c r="G12" t="s">
-        <v>314</v>
-      </c>
       <c r="H12" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -4197,13 +4217,13 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G13" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H13" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -4214,13 +4234,13 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G14" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H14" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -4231,22 +4251,22 @@
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D15" t="s">
+        <v>314</v>
+      </c>
+      <c r="E15" t="s">
+        <v>315</v>
+      </c>
+      <c r="F15" t="s">
         <v>316</v>
       </c>
-      <c r="E15" t="s">
+      <c r="G15" t="s">
         <v>317</v>
       </c>
-      <c r="F15" t="s">
-        <v>318</v>
-      </c>
-      <c r="G15" t="s">
-        <v>319</v>
-      </c>
       <c r="H15" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -4257,22 +4277,22 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D16" t="s">
+        <v>318</v>
+      </c>
+      <c r="E16" t="s">
+        <v>319</v>
+      </c>
+      <c r="F16" t="s">
         <v>320</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>321</v>
       </c>
-      <c r="F16" t="s">
-        <v>322</v>
-      </c>
-      <c r="G16" t="s">
-        <v>323</v>
-      </c>
       <c r="H16" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -4283,13 +4303,13 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G17" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H17" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -4300,13 +4320,13 @@
         <v>3</v>
       </c>
       <c r="C18" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G18" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H18" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -4317,22 +4337,22 @@
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D19" t="s">
+        <v>324</v>
+      </c>
+      <c r="E19" t="s">
+        <v>325</v>
+      </c>
+      <c r="F19" t="s">
         <v>326</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" t="s">
         <v>327</v>
       </c>
-      <c r="F19" t="s">
-        <v>328</v>
-      </c>
-      <c r="G19" t="s">
-        <v>329</v>
-      </c>
       <c r="H19" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -4343,22 +4363,22 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D20" t="s">
+        <v>328</v>
+      </c>
+      <c r="E20" t="s">
+        <v>329</v>
+      </c>
+      <c r="F20" t="s">
         <v>330</v>
       </c>
-      <c r="E20" t="s">
+      <c r="G20" t="s">
         <v>331</v>
       </c>
-      <c r="F20" t="s">
-        <v>332</v>
-      </c>
-      <c r="G20" t="s">
-        <v>333</v>
-      </c>
       <c r="H20" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -4369,13 +4389,13 @@
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G21" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H21" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -4386,13 +4406,13 @@
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G22" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="H22" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -4403,13 +4423,13 @@
         <v>4</v>
       </c>
       <c r="C23" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G23" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="H23" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -4420,22 +4440,22 @@
         <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D24" t="s">
+        <v>335</v>
+      </c>
+      <c r="E24" t="s">
+        <v>336</v>
+      </c>
+      <c r="F24" t="s">
+        <v>330</v>
+      </c>
+      <c r="G24" t="s">
         <v>337</v>
       </c>
-      <c r="E24" t="s">
-        <v>338</v>
-      </c>
-      <c r="F24" t="s">
-        <v>332</v>
-      </c>
-      <c r="G24" t="s">
-        <v>339</v>
-      </c>
       <c r="H24" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -4446,22 +4466,22 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D25" t="s">
+        <v>338</v>
+      </c>
+      <c r="E25" t="s">
+        <v>339</v>
+      </c>
+      <c r="F25" t="s">
         <v>340</v>
       </c>
-      <c r="E25" t="s">
+      <c r="G25" t="s">
         <v>341</v>
       </c>
-      <c r="F25" t="s">
-        <v>342</v>
-      </c>
-      <c r="G25" t="s">
-        <v>343</v>
-      </c>
       <c r="H25" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -4472,13 +4492,13 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G26" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H26" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -4489,13 +4509,13 @@
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G27" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H27" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -4506,13 +4526,13 @@
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G28" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H28" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -4523,22 +4543,22 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D29" t="s">
+        <v>342</v>
+      </c>
+      <c r="E29" t="s">
+        <v>343</v>
+      </c>
+      <c r="F29" t="s">
         <v>344</v>
       </c>
-      <c r="E29" t="s">
+      <c r="G29" t="s">
         <v>345</v>
       </c>
-      <c r="F29" t="s">
-        <v>346</v>
-      </c>
-      <c r="G29" t="s">
-        <v>347</v>
-      </c>
       <c r="H29" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -4549,22 +4569,22 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D30" t="s">
+        <v>346</v>
+      </c>
+      <c r="E30" t="s">
+        <v>347</v>
+      </c>
+      <c r="F30" t="s">
         <v>348</v>
       </c>
-      <c r="E30" t="s">
+      <c r="G30" t="s">
         <v>349</v>
       </c>
-      <c r="F30" t="s">
-        <v>350</v>
-      </c>
-      <c r="G30" t="s">
-        <v>351</v>
-      </c>
       <c r="H30" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -4575,13 +4595,13 @@
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G31" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H31" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -4592,13 +4612,13 @@
         <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G32" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H32" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -4609,13 +4629,13 @@
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G33" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H33" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -4626,22 +4646,22 @@
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D34" t="s">
+        <v>352</v>
+      </c>
+      <c r="E34" t="s">
+        <v>353</v>
+      </c>
+      <c r="F34" t="s">
         <v>354</v>
       </c>
-      <c r="E34" t="s">
+      <c r="G34" t="s">
         <v>355</v>
       </c>
-      <c r="F34" t="s">
-        <v>356</v>
-      </c>
-      <c r="G34" t="s">
-        <v>357</v>
-      </c>
       <c r="H34" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -4652,22 +4672,22 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D35" t="s">
+        <v>356</v>
+      </c>
+      <c r="E35" t="s">
+        <v>357</v>
+      </c>
+      <c r="F35" t="s">
         <v>358</v>
       </c>
-      <c r="E35" t="s">
+      <c r="G35" t="s">
         <v>359</v>
       </c>
-      <c r="F35" t="s">
-        <v>360</v>
-      </c>
-      <c r="G35" t="s">
-        <v>361</v>
-      </c>
       <c r="H35" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -4678,13 +4698,13 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G36" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H36" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -4695,13 +4715,13 @@
         <v>3</v>
       </c>
       <c r="C37" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G37" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H37" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -4712,13 +4732,13 @@
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G38" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H38" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -4729,22 +4749,22 @@
         <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D39" t="s">
+        <v>360</v>
+      </c>
+      <c r="E39" t="s">
+        <v>361</v>
+      </c>
+      <c r="F39" t="s">
         <v>362</v>
       </c>
-      <c r="E39" t="s">
+      <c r="G39" t="s">
         <v>363</v>
       </c>
-      <c r="F39" t="s">
-        <v>364</v>
-      </c>
-      <c r="G39" t="s">
-        <v>365</v>
-      </c>
       <c r="H39" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -4755,22 +4775,22 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D40" t="s">
+        <v>356</v>
+      </c>
+      <c r="E40" t="s">
+        <v>357</v>
+      </c>
+      <c r="F40" t="s">
         <v>358</v>
       </c>
-      <c r="E40" t="s">
+      <c r="G40" t="s">
         <v>359</v>
       </c>
-      <c r="F40" t="s">
-        <v>360</v>
-      </c>
-      <c r="G40" t="s">
-        <v>361</v>
-      </c>
       <c r="H40" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -4781,13 +4801,13 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G41" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H41" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -4798,13 +4818,13 @@
         <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G42" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H42" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -4815,13 +4835,13 @@
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G43" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H43" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -4832,22 +4852,22 @@
         <v>5</v>
       </c>
       <c r="C44" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D44" t="s">
+        <v>360</v>
+      </c>
+      <c r="E44" t="s">
+        <v>361</v>
+      </c>
+      <c r="F44" t="s">
         <v>362</v>
       </c>
-      <c r="E44" t="s">
+      <c r="G44" t="s">
         <v>363</v>
       </c>
-      <c r="F44" t="s">
-        <v>364</v>
-      </c>
-      <c r="G44" t="s">
-        <v>365</v>
-      </c>
       <c r="H44" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -4858,22 +4878,22 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D45" t="s">
+        <v>364</v>
+      </c>
+      <c r="E45" t="s">
+        <v>365</v>
+      </c>
+      <c r="F45" t="s">
         <v>366</v>
       </c>
-      <c r="E45" t="s">
+      <c r="G45" t="s">
         <v>367</v>
       </c>
-      <c r="F45" t="s">
-        <v>368</v>
-      </c>
-      <c r="G45" t="s">
-        <v>369</v>
-      </c>
       <c r="H45" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -4884,13 +4904,13 @@
         <v>2</v>
       </c>
       <c r="C46" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G46" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H46" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -4901,13 +4921,13 @@
         <v>3</v>
       </c>
       <c r="C47" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G47" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H47" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -4918,13 +4938,13 @@
         <v>4</v>
       </c>
       <c r="C48" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G48" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H48" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -4935,22 +4955,22 @@
         <v>5</v>
       </c>
       <c r="C49" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D49" t="s">
+        <v>368</v>
+      </c>
+      <c r="E49" t="s">
+        <v>369</v>
+      </c>
+      <c r="F49" t="s">
         <v>370</v>
       </c>
-      <c r="E49" t="s">
+      <c r="G49" t="s">
         <v>371</v>
       </c>
-      <c r="F49" t="s">
-        <v>372</v>
-      </c>
-      <c r="G49" t="s">
-        <v>373</v>
-      </c>
       <c r="H49" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -4961,22 +4981,22 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D50" t="s">
+        <v>372</v>
+      </c>
+      <c r="E50" t="s">
+        <v>373</v>
+      </c>
+      <c r="F50" t="s">
         <v>374</v>
       </c>
-      <c r="E50" t="s">
+      <c r="G50" t="s">
         <v>375</v>
       </c>
-      <c r="F50" t="s">
-        <v>376</v>
-      </c>
-      <c r="G50" t="s">
-        <v>377</v>
-      </c>
       <c r="H50" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -4987,13 +5007,13 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G51" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H51" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -5004,13 +5024,13 @@
         <v>3</v>
       </c>
       <c r="C52" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G52" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H52" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -5021,13 +5041,13 @@
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G53" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H53" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -5038,22 +5058,22 @@
         <v>5</v>
       </c>
       <c r="C54" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D54" t="s">
+        <v>376</v>
+      </c>
+      <c r="E54" t="s">
+        <v>377</v>
+      </c>
+      <c r="F54" t="s">
         <v>378</v>
       </c>
-      <c r="E54" t="s">
+      <c r="G54" t="s">
         <v>379</v>
       </c>
-      <c r="F54" t="s">
-        <v>380</v>
-      </c>
-      <c r="G54" t="s">
-        <v>381</v>
-      </c>
       <c r="H54" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -5064,22 +5084,22 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D55" t="s">
+        <v>380</v>
+      </c>
+      <c r="E55" t="s">
+        <v>381</v>
+      </c>
+      <c r="F55" t="s">
         <v>382</v>
       </c>
-      <c r="E55" t="s">
+      <c r="G55" t="s">
         <v>383</v>
       </c>
-      <c r="F55" t="s">
-        <v>384</v>
-      </c>
-      <c r="G55" t="s">
-        <v>385</v>
-      </c>
       <c r="H55" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -5090,22 +5110,22 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D56" t="s">
+        <v>384</v>
+      </c>
+      <c r="E56" t="s">
+        <v>385</v>
+      </c>
+      <c r="F56" t="s">
         <v>386</v>
       </c>
-      <c r="E56" t="s">
+      <c r="G56" t="s">
         <v>387</v>
       </c>
-      <c r="F56" t="s">
-        <v>388</v>
-      </c>
-      <c r="G56" t="s">
-        <v>389</v>
-      </c>
       <c r="H56" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -5116,13 +5136,13 @@
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G57" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H57" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -5133,13 +5153,13 @@
         <v>3</v>
       </c>
       <c r="C58" t="s">
+        <v>301</v>
+      </c>
+      <c r="G58" t="s">
         <v>303</v>
       </c>
-      <c r="G58" t="s">
-        <v>305</v>
-      </c>
       <c r="H58" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -5150,13 +5170,13 @@
         <v>4</v>
       </c>
       <c r="C59" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G59" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H59" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -5167,22 +5187,22 @@
         <v>5</v>
       </c>
       <c r="C60" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D60" t="s">
+        <v>388</v>
+      </c>
+      <c r="E60" t="s">
+        <v>389</v>
+      </c>
+      <c r="F60" t="s">
         <v>390</v>
       </c>
-      <c r="E60" t="s">
+      <c r="G60" t="s">
         <v>391</v>
       </c>
-      <c r="F60" t="s">
-        <v>392</v>
-      </c>
-      <c r="G60" t="s">
-        <v>393</v>
-      </c>
       <c r="H60" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -5193,22 +5213,22 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D61" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E61" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="F61" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G61" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="H61" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -5219,13 +5239,13 @@
         <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G62" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H62" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -5236,13 +5256,13 @@
         <v>3</v>
       </c>
       <c r="C63" t="s">
+        <v>301</v>
+      </c>
+      <c r="G63" t="s">
         <v>303</v>
       </c>
-      <c r="G63" t="s">
-        <v>305</v>
-      </c>
       <c r="H63" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -5253,13 +5273,13 @@
         <v>4</v>
       </c>
       <c r="C64" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G64" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="H64" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -5270,22 +5290,22 @@
         <v>5</v>
       </c>
       <c r="C65" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D65" t="s">
+        <v>394</v>
+      </c>
+      <c r="E65" t="s">
+        <v>395</v>
+      </c>
+      <c r="F65" t="s">
         <v>396</v>
       </c>
-      <c r="E65" t="s">
+      <c r="G65" t="s">
         <v>397</v>
       </c>
-      <c r="F65" t="s">
-        <v>398</v>
-      </c>
-      <c r="G65" t="s">
-        <v>399</v>
-      </c>
       <c r="H65" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -5296,22 +5316,22 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D66" t="s">
+        <v>398</v>
+      </c>
+      <c r="E66" t="s">
+        <v>399</v>
+      </c>
+      <c r="F66" t="s">
         <v>400</v>
       </c>
-      <c r="E66" t="s">
+      <c r="G66" t="s">
         <v>401</v>
       </c>
-      <c r="F66" t="s">
-        <v>402</v>
-      </c>
-      <c r="G66" t="s">
-        <v>403</v>
-      </c>
       <c r="H66" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -5322,13 +5342,13 @@
         <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G67" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H67" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -5339,13 +5359,13 @@
         <v>3</v>
       </c>
       <c r="C68" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G68" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H68" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -5356,13 +5376,13 @@
         <v>4</v>
       </c>
       <c r="C69" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G69" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H69" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -5373,19 +5393,19 @@
         <v>5</v>
       </c>
       <c r="C70" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="E70" t="s">
+        <v>403</v>
+      </c>
+      <c r="F70" t="s">
+        <v>404</v>
+      </c>
+      <c r="G70" t="s">
         <v>405</v>
       </c>
-      <c r="F70" t="s">
-        <v>406</v>
-      </c>
-      <c r="G70" t="s">
-        <v>407</v>
-      </c>
       <c r="H70" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -5396,13 +5416,13 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="G71" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="H71" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>